<commit_message>
Updated the input files for the Differential analysis
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\swains\Desktop\IGBMC\ASO_ShRNA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\swains\Desktop\IGBMC\ASO_ShRNA\STIM1therORAI1_LPG_SPS26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E014427-2C40-49E3-BC5F-0FDF093A7E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BDDDA9F-7F5D-4881-9F6E-10A78CB8BC54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{51D6F311-4D22-44C5-8915-D345C9BC7C00}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
   <si>
     <t>sample</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>KZLX8</t>
-  </si>
-  <si>
-    <t>KZLX9</t>
   </si>
   <si>
     <t>KZLX10</t>
@@ -700,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCC58352-B0E8-475D-A789-69640F573AB9}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.5546875" customWidth="1"/>
@@ -719,7 +716,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -727,7 +724,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -735,7 +732,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -743,7 +740,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -751,7 +748,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -759,7 +756,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -767,7 +764,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -775,7 +772,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -783,7 +780,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -791,7 +788,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -799,15 +796,15 @@
         <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>31</v>
+      <c r="B13" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -815,7 +812,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -823,7 +820,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -831,15 +828,15 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
-      <c r="B17" t="s">
-        <v>29</v>
+      <c r="B17" s="2" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -847,7 +844,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -855,7 +852,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -863,15 +860,15 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>27</v>
+      <c r="B21" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -879,7 +876,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -887,7 +884,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -895,15 +892,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>